<commit_message>
Tweak to epix™ Pro
</commit_message>
<xml_diff>
--- a/data/raw/xlsx/concise.xlsx
+++ b/data/raw/xlsx/concise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mike\projects\work\garmin-ids\data\raw\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9EE7871-1BA5-466F-982C-B40472C61B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD47C49-37DD-4415-B577-FE3E987D9F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5504BBCC-0CF3-4847-80C4-174D6616E638}"/>
   </bookViews>
@@ -635,9 +635,6 @@
     <t>Part</t>
   </si>
   <si>
-    <t>epix™ Pro (Gen 2) - 47 mm / quatix® 7 Pro</t>
-  </si>
-  <si>
     <t>ForeAthlete® 45 / 45S</t>
   </si>
   <si>
@@ -648,6 +645,9 @@
   </si>
   <si>
     <t>ForeAthlete® 55 / Forerunner® 158</t>
+  </si>
+  <si>
+    <t>epix™ Pro - 47 mm / quatix® 7 Pro</t>
   </si>
 </sst>
 </file>
@@ -1155,7 +1155,7 @@
         <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>24</v>
@@ -1169,7 +1169,7 @@
         <v>26</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>27</v>
@@ -1437,7 +1437,7 @@
         <v>77</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>78</v>
@@ -1723,7 +1723,7 @@
         <v>141</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>142</v>
@@ -1737,7 +1737,7 @@
         <v>144</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>145</v>

</xml_diff>